<commit_message>
fix: corrige nome do indicador de valor medio por unidade
</commit_message>
<xml_diff>
--- a/saida/relatorio_automatizado.xlsx
+++ b/saida/relatorio_automatizado.xlsx
@@ -490,7 +490,7 @@
         <v>126.2</v>
       </c>
       <c r="G2" t="n">
-        <v>21.03333333333333</v>
+        <v>21.03</v>
       </c>
     </row>
     <row r="3">
@@ -568,10 +568,10 @@
         <v>20.56</v>
       </c>
       <c r="F5" t="n">
-        <v>108.04</v>
+        <v>87.48</v>
       </c>
       <c r="G5" t="n">
-        <v>22.30666666666667</v>
+        <v>29.16</v>
       </c>
     </row>
     <row r="6">
@@ -595,10 +595,10 @@
         <v>51.32</v>
       </c>
       <c r="F6" t="n">
-        <v>606.5</v>
+        <v>555.1799999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>27.99222222222222</v>
+        <v>30.84</v>
       </c>
     </row>
     <row r="7">
@@ -622,10 +622,10 @@
         <v>139.52</v>
       </c>
       <c r="F7" t="n">
-        <v>2771.77</v>
+        <v>2632.25</v>
       </c>
       <c r="G7" t="n">
-        <v>31.95807692307692</v>
+        <v>33.75</v>
       </c>
     </row>
     <row r="8">
@@ -649,10 +649,10 @@
         <v>0.99</v>
       </c>
       <c r="F8" t="n">
-        <v>92.50999999999999</v>
+        <v>91.52</v>
       </c>
       <c r="G8" t="n">
-        <v>30.17666666666667</v>
+        <v>30.51</v>
       </c>
     </row>
   </sheetData>
@@ -684,7 +684,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Total de vendas</t>
+          <t>Total de Vendas</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -694,7 +694,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Valor dos produtos</t>
+          <t>Valor dos Produtos</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -704,7 +704,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Total de frete</t>
+          <t>Total de Frete</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -714,21 +714,21 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Total geral</t>
+          <t>Total Geral</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3764.17</v>
+        <v>3551.78</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ticket médio</t>
+          <t>Valor Médio por Unidade (c/ Frete)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>34.21972727272728</v>
+        <v>32.29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>